<commit_message>
feat(user-reports): add 433-ek Excel sanawy and ministry placeholders
Add 433-ek.xlsx seed (15-column sanawy), update gurlusyk placeholders, and ApplicationItem fields for education/visa/foreign address. Remove unused Personnel_List_Seed. ExcelTemplateSpike can build 433-ek from source .xls.
</commit_message>
<xml_diff>
--- a/Visa2026.Module/Resources/Templates/Excel/gurlusyk_uzt.xlsx
+++ b/Visa2026.Module/Resources/Templates/Excel/gurlusyk_uzt.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webap\Documents\GitHub\Visa2026\Visa2026.Module\Resources\Templates\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A752E6B-D792-4CEF-A978-476B7A31F1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382344DA-82E8-4AE0-91EA-8471BB6F0354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{D1924FAF-F3EB-4137-A933-DEF56DEDE6ED}"/>
   </bookViews>
@@ -23,59 +23,53 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
-  <si>
-    <t>№</t>
-  </si>
-  <si>
-    <t>Familiýasy</t>
-  </si>
-  <si>
-    <t>Ady</t>
-  </si>
-  <si>
-    <t>Doglan senesi we ýeri</t>
-  </si>
-  <si>
-    <t>Jynsy</t>
-  </si>
-  <si>
-    <t>Raýatlygy</t>
-  </si>
-  <si>
-    <t>Pasport belgisi we möhleti</t>
-  </si>
-  <si>
-    <t>Bilimi we okan ýeri</t>
-  </si>
-  <si>
-    <t>Bilimine görä hünäri</t>
-  </si>
-  <si>
-    <t>Wezipesi</t>
-  </si>
-  <si>
-    <t>Möhleti we gezekligi</t>
-  </si>
-  <si>
-    <t>Gelmeginiň maksady</t>
-  </si>
-  <si>
-    <t>Çagyrýan Tarap</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+  <si>
+    <t xml:space="preserve">                                                                                                                                  Türkmenistanyň Energetika Ministrligi
+                                                                                                                 “         ”  “       ” 2026-nji ýylyň                    belgili hatynyň 1 belgili goşundysy</t>
   </si>
   <si>
     <t xml:space="preserve">                                                                                                         Ylalaşylan daşary ýurt raýatlarynyň
                                                                                                                         SANAWY</t>
   </si>
   <si>
-    <t xml:space="preserve">                                                                      Ministr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                  A.Saparow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                                                                                  Türkmenistanyň Energetika Ministrligi
-                                                                                                                 “         ”  “       ” 2026-nji ýylyň                    belgili hatynyň 1 belgili goşundysy</t>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Familiýasy</t>
+  </si>
+  <si>
+    <t>Ady</t>
+  </si>
+  <si>
+    <t>Doglan senesi we ýeri</t>
+  </si>
+  <si>
+    <t>Jynsy</t>
+  </si>
+  <si>
+    <t>Raýatlygy</t>
+  </si>
+  <si>
+    <t>Pasport belgisi we möhleti</t>
+  </si>
+  <si>
+    <t>Bilimi we okan ýeri</t>
+  </si>
+  <si>
+    <t>Bilimine görä hünäri</t>
+  </si>
+  <si>
+    <t>Wezipesi</t>
+  </si>
+  <si>
+    <t>Gelmeginiň maksady</t>
+  </si>
+  <si>
+    <t>Çagyrýan Tarap</t>
+  </si>
+  <si>
+    <t>Möhleti we gezekligi</t>
   </si>
   <si>
     <t>{{#ds.rows}}</t>
@@ -106,7 +100,7 @@
   </si>
   <si>
     <t xml:space="preserve">	
-{{.Education_LevelTm}}</t>
+{{.Education_LevelAndInstitutionTm}}</t>
   </si>
   <si>
     <t>{{.Education_SpecialtyTm}}</t>
@@ -121,13 +115,22 @@
   </si>
   <si>
     <t>{{.Application_SponsorName}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                      Ministr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                  A.Saparow</t>
+  </si>
+  <si>
+    <t>{{.Visa_DurationFrequencyBlock}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -194,12 +197,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -326,12 +323,6 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -341,6 +332,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -352,15 +358,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -644,8 +641,8 @@
   <cols>
     <col min="1" max="1" width="0.7109375" customWidth="1"/>
     <col min="2" max="2" width="10" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="7" customWidth="1"/>
     <col min="5" max="5" width="14.140625" style="7" customWidth="1"/>
     <col min="6" max="6" width="13.140625" style="7" customWidth="1"/>
     <col min="7" max="7" width="14" style="7" customWidth="1"/>
@@ -658,6 +655,7 @@
     <col min="15" max="15" width="14.5703125" style="5" customWidth="1"/>
     <col min="16" max="16" width="13.5703125" style="5" customWidth="1"/>
     <col min="17" max="17" width="56" customWidth="1"/>
+    <col min="18" max="19" width="9.140625" customWidth="1"/>
     <col min="20" max="20" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -665,174 +663,176 @@
       <c r="D1" s="4"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
+      <c r="G1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
     </row>
     <row r="2" spans="3:16" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D2" s="4"/>
-      <c r="E2" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
+      <c r="E2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
     </row>
     <row r="3" spans="3:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D3" s="6" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="3:16" ht="178.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="G4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="H4" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="I4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="J4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="K4" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="L4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="M4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="N4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="P4" s="13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="3:16" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="10"/>
-    </row>
-    <row r="5" spans="3:16" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
     </row>
     <row r="6" spans="3:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
     </row>
     <row r="7" spans="3:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
     </row>
     <row r="8" spans="3:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
     </row>
     <row r="12" spans="3:16" x14ac:dyDescent="0.25">
       <c r="G12" s="8"/>
@@ -848,10 +848,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="G1:P1"/>
+    <mergeCell ref="E2:P2"/>
     <mergeCell ref="E5:K8"/>
     <mergeCell ref="L5:O8"/>
-    <mergeCell ref="G1:P1"/>
-    <mergeCell ref="E2:P2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.17" right="0.17" top="0.25" bottom="0.32" header="0.17" footer="0.3"/>

</xml_diff>